<commit_message>
Se añade análisis de perdida/ganancia en venta de acciones
</commit_message>
<xml_diff>
--- a/documentacion/SIPRO_TO_DO.xlsx
+++ b/documentacion/SIPRO_TO_DO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PROYECTOS\SIPRO_07\documentacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0286F970-CDCF-420B-B473-7B3160299F65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62C7D8FF-E728-47E5-98A8-2B78747B01A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -534,15 +534,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>68035</xdr:colOff>
-      <xdr:row>51</xdr:row>
-      <xdr:rowOff>76541</xdr:rowOff>
+      <xdr:colOff>110557</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>93550</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>3925178</xdr:colOff>
-      <xdr:row>69</xdr:row>
-      <xdr:rowOff>80202</xdr:rowOff>
+      <xdr:colOff>3967700</xdr:colOff>
+      <xdr:row>58</xdr:row>
+      <xdr:rowOff>97212</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -565,7 +565,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1250156" y="3648416"/>
+          <a:off x="1292678" y="4975113"/>
           <a:ext cx="3857143" cy="3371429"/>
         </a:xfrm>
         <a:prstGeom prst="rect">

</xml_diff>

<commit_message>
antes de analizar Bolsa de Valores de Guayaquil
</commit_message>
<xml_diff>
--- a/documentacion/SIPRO_TO_DO.xlsx
+++ b/documentacion/SIPRO_TO_DO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PROYECTOS\SIPRO_07\documentacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62C7D8FF-E728-47E5-98A8-2B78747B01A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{621CC4CD-BDC6-43E2-8281-D481FD3F8ED4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="68">
   <si>
     <t>Implementar registro de acciones</t>
   </si>
@@ -328,6 +328,27 @@
   </si>
   <si>
     <t>Investigar como automatizar cosas con Power Automate</t>
+  </si>
+  <si>
+    <t>Automatizacion</t>
+  </si>
+  <si>
+    <t>Personal</t>
+  </si>
+  <si>
+    <t>CargaDiaria</t>
+  </si>
+  <si>
+    <t>Crear interfaz de analisis de archivos descargados</t>
+  </si>
+  <si>
+    <t>Carga de datos de archivos diarios de BVQ desde el sistema</t>
+  </si>
+  <si>
+    <t>Carga de datos de archivos diarios de BVG desde el sistema</t>
+  </si>
+  <si>
+    <t>Crear funcionalidad de descarga de Ofertas y Demandas a las 4:30</t>
   </si>
 </sst>
 </file>
@@ -393,7 +414,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -414,17 +435,6 @@
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
       <diagonal/>
     </border>
   </borders>
@@ -459,8 +469,8 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -487,13 +497,13 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>51</xdr:row>
+      <xdr:row>58</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
-      <xdr:row>52</xdr:row>
+      <xdr:row>59</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -535,14 +545,14 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>110557</xdr:colOff>
-      <xdr:row>40</xdr:row>
+      <xdr:row>47</xdr:row>
       <xdr:rowOff>93550</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
       <xdr:colOff>3967700</xdr:colOff>
-      <xdr:row>58</xdr:row>
-      <xdr:rowOff>97212</xdr:rowOff>
+      <xdr:row>65</xdr:row>
+      <xdr:rowOff>97211</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -889,11 +899,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
-  <dimension ref="A1:G70"/>
+  <dimension ref="A1:G77"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="133.5703125" style="6" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="17.140625" bestFit="1" customWidth="1"/>
@@ -924,7 +933,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -947,7 +956,7 @@
         <v>46194</v>
       </c>
     </row>
-    <row r="3" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -970,7 +979,7 @@
         <v>46207</v>
       </c>
     </row>
-    <row r="4" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -1014,7 +1023,7 @@
       </c>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -1037,7 +1046,7 @@
         <v>46207</v>
       </c>
     </row>
-    <row r="7" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -1060,7 +1069,7 @@
         <v>46249</v>
       </c>
     </row>
-    <row r="8" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -1081,7 +1090,7 @@
       </c>
       <c r="G8" s="2"/>
     </row>
-    <row r="9" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -1102,7 +1111,7 @@
       </c>
       <c r="G9" s="2"/>
     </row>
-    <row r="10" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -1146,7 +1155,7 @@
       </c>
       <c r="G11" s="2"/>
     </row>
-    <row r="12" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -1169,7 +1178,7 @@
         <v>46200</v>
       </c>
     </row>
-    <row r="13" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>12</v>
       </c>
@@ -1192,7 +1201,7 @@
         <v>46207</v>
       </c>
     </row>
-    <row r="14" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>13</v>
       </c>
@@ -1215,7 +1224,7 @@
         <v>46207</v>
       </c>
     </row>
-    <row r="15" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>14</v>
       </c>
@@ -1238,7 +1247,7 @@
         <v>46249</v>
       </c>
     </row>
-    <row r="16" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>15</v>
       </c>
@@ -1261,7 +1270,7 @@
         <v>46207</v>
       </c>
     </row>
-    <row r="17" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <v>16</v>
       </c>
@@ -1305,9 +1314,9 @@
       </c>
       <c r="G18" s="2"/>
     </row>
-    <row r="19" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>23</v>
@@ -1328,9 +1337,9 @@
         <v>46249</v>
       </c>
     </row>
-    <row r="20" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>14</v>
@@ -1353,7 +1362,7 @@
     </row>
     <row r="21" spans="1:7" ht="75" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>36</v>
@@ -1372,9 +1381,9 @@
       </c>
       <c r="G21" s="2"/>
     </row>
-    <row r="22" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="2">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>15</v>
@@ -1395,9 +1404,9 @@
         <v>46250</v>
       </c>
     </row>
-    <row r="23" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="2">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>18</v>
@@ -1420,7 +1429,7 @@
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="2">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>36</v>
@@ -1441,7 +1450,7 @@
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="2">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>36</v>
@@ -1462,7 +1471,7 @@
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="2">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>36</v>
@@ -1483,7 +1492,7 @@
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="2">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B27" s="2" t="s">
         <v>14</v>
@@ -1503,13 +1512,13 @@
       <c r="G27" s="2"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="12">
+      <c r="A28" s="2">
         <v>27</v>
       </c>
-      <c r="B28" s="12" t="s">
+      <c r="B28" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C28" s="6" t="s">
+      <c r="C28" s="5" t="s">
         <v>57</v>
       </c>
       <c r="D28" s="2">
@@ -1521,90 +1530,216 @@
       <c r="F28" s="3">
         <v>46255</v>
       </c>
+      <c r="G28" s="2"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C29" s="6" t="s">
+      <c r="A29" s="2">
+        <v>28</v>
+      </c>
+      <c r="B29" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="C29" s="5" t="s">
         <v>58</v>
       </c>
+      <c r="D29" s="2">
+        <v>1</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F29" s="3">
+        <v>46285</v>
+      </c>
+      <c r="G29" s="2"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30" s="2">
+        <v>29</v>
+      </c>
+      <c r="B30" s="12" t="s">
+        <v>61</v>
+      </c>
       <c r="C30" s="5" t="s">
         <v>60</v>
       </c>
+      <c r="D30" s="2">
+        <v>1</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F30" s="3">
+        <v>46285</v>
+      </c>
+      <c r="G30" s="2"/>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31" s="2">
+        <v>30</v>
+      </c>
+      <c r="B31" s="12" t="s">
+        <v>62</v>
+      </c>
       <c r="C31" s="13" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="51" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="E51">
+      <c r="D31" s="2">
+        <v>1</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F31" s="3">
+        <v>46285</v>
+      </c>
+      <c r="G31" s="2"/>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32" s="2">
+        <v>31</v>
+      </c>
+      <c r="B32" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D32" s="2">
+        <v>1</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F32" s="3">
+        <v>46285</v>
+      </c>
+      <c r="G32" s="2"/>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33" s="2">
+        <v>32</v>
+      </c>
+      <c r="B33" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="D33" s="2">
+        <v>1</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F33" s="3">
+        <v>46293</v>
+      </c>
+      <c r="G33" s="2"/>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" s="2">
+        <v>33</v>
+      </c>
+      <c r="B34" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="C34" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="D34" s="2">
+        <v>1</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F34" s="3">
+        <v>46293</v>
+      </c>
+      <c r="G34" s="2"/>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" s="2">
+        <v>34</v>
+      </c>
+      <c r="B35" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="C35" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="D35" s="2">
+        <v>1</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F35" s="3">
+        <v>46293</v>
+      </c>
+      <c r="G35" s="2"/>
+    </row>
+    <row r="58" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="E58">
         <v>28401.05</v>
       </c>
     </row>
-    <row r="52" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C52"/>
-      <c r="E52" s="7">
+    <row r="59" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="C59"/>
+      <c r="E59" s="7">
         <v>28374.3</v>
       </c>
     </row>
-    <row r="53" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="E53">
-        <f>E51-E52</f>
+    <row r="60" spans="3:5" x14ac:dyDescent="0.25">
+      <c r="E60">
+        <f>E58-E59</f>
         <v>26.75</v>
       </c>
     </row>
-    <row r="58" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="E58" t="s">
+    <row r="65" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="E65" t="s">
         <v>44</v>
       </c>
-      <c r="F58">
+      <c r="F65">
         <v>696</v>
       </c>
     </row>
-    <row r="59" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="E59" t="s">
+    <row r="66" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="E66" t="s">
         <v>45</v>
       </c>
-      <c r="F59">
+      <c r="F66">
         <v>146</v>
       </c>
     </row>
-    <row r="62" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="E62">
+    <row r="69" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="E69">
         <v>752.79</v>
       </c>
-      <c r="F62">
+      <c r="F69">
         <v>26.75</v>
       </c>
     </row>
-    <row r="63" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="E63">
+    <row r="70" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="E70">
         <v>100</v>
       </c>
-      <c r="F63">
-        <f>E63*F62/E62</f>
+      <c r="F70">
+        <f>E70*F69/E69</f>
         <v>3.5534478406992656</v>
       </c>
     </row>
-    <row r="68" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C68" s="6" t="s">
+    <row r="75" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C75" s="6" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="70" spans="3:3" x14ac:dyDescent="0.25">
-      <c r="C70" s="6" t="s">
+    <row r="77" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C77" s="6" t="s">
         <v>38</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G29" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="4">
-      <filters blank="1">
-        <filter val="Pendiente"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
   <hyperlinks>
     <hyperlink ref="C31" r:id="rId1" xr:uid="{3C22A885-07EB-43DB-A866-EAD7FAA5DC07}"/>
   </hyperlinks>

</xml_diff>

<commit_message>
Primera version descarga de Archivos de BVG
</commit_message>
<xml_diff>
--- a/documentacion/SIPRO_TO_DO.xlsx
+++ b/documentacion/SIPRO_TO_DO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PROYECTOS\SIPRO_07\documentacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{621CC4CD-BDC6-43E2-8281-D481FD3F8ED4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58923BF5-3B22-40AE-A916-AFB089C80454}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="67">
   <si>
     <t>Implementar registro de acciones</t>
   </si>
@@ -343,9 +343,6 @@
   </si>
   <si>
     <t>Carga de datos de archivos diarios de BVQ desde el sistema</t>
-  </si>
-  <si>
-    <t>Carga de datos de archivos diarios de BVG desde el sistema</t>
   </si>
   <si>
     <t>Crear funcionalidad de descarga de Ofertas y Demandas a las 4:30</t>
@@ -442,7 +439,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -469,7 +466,6 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -497,13 +493,13 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>58</xdr:row>
+      <xdr:row>57</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
-      <xdr:row>59</xdr:row>
+      <xdr:row>58</xdr:row>
       <xdr:rowOff>114300</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
@@ -545,13 +541,13 @@
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>110557</xdr:colOff>
-      <xdr:row>47</xdr:row>
+      <xdr:row>46</xdr:row>
       <xdr:rowOff>93550</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
       <xdr:colOff>3967700</xdr:colOff>
-      <xdr:row>65</xdr:row>
+      <xdr:row>64</xdr:row>
       <xdr:rowOff>97211</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -899,7 +895,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G77"/>
+  <dimension ref="A1:G76"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" bestFit="1" customWidth="1"/>
@@ -1536,7 +1532,7 @@
       <c r="A29" s="2">
         <v>28</v>
       </c>
-      <c r="B29" s="12" t="s">
+      <c r="B29" s="2" t="s">
         <v>61</v>
       </c>
       <c r="C29" s="5" t="s">
@@ -1557,7 +1553,7 @@
       <c r="A30" s="2">
         <v>29</v>
       </c>
-      <c r="B30" s="12" t="s">
+      <c r="B30" s="2" t="s">
         <v>61</v>
       </c>
       <c r="C30" s="5" t="s">
@@ -1578,10 +1574,10 @@
       <c r="A31" s="2">
         <v>30</v>
       </c>
-      <c r="B31" s="12" t="s">
+      <c r="B31" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="C31" s="13" t="s">
+      <c r="C31" s="12" t="s">
         <v>59</v>
       </c>
       <c r="D31" s="2">
@@ -1599,7 +1595,7 @@
       <c r="A32" s="2">
         <v>31</v>
       </c>
-      <c r="B32" s="12" t="s">
+      <c r="B32" s="2" t="s">
         <v>63</v>
       </c>
       <c r="C32" s="5" t="s">
@@ -1620,11 +1616,11 @@
       <c r="A33" s="2">
         <v>32</v>
       </c>
-      <c r="B33" s="12" t="s">
+      <c r="B33" s="2" t="s">
         <v>63</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D33" s="2">
         <v>1</v>
@@ -1641,11 +1637,11 @@
       <c r="A34" s="2">
         <v>33</v>
       </c>
-      <c r="B34" s="12" t="s">
+      <c r="B34" s="2" t="s">
         <v>63</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D34" s="2">
         <v>1</v>
@@ -1658,84 +1654,63 @@
       </c>
       <c r="G34" s="2"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A35" s="2">
-        <v>34</v>
-      </c>
-      <c r="B35" s="12" t="s">
-        <v>63</v>
-      </c>
-      <c r="C35" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="D35" s="2">
-        <v>1</v>
-      </c>
-      <c r="E35" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="F35" s="3">
-        <v>46293</v>
-      </c>
-      <c r="G35" s="2"/>
-    </row>
-    <row r="58" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E58">
+    <row r="57" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="E57">
         <v>28401.05</v>
       </c>
     </row>
-    <row r="59" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="C59"/>
-      <c r="E59" s="7">
+    <row r="58" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C58"/>
+      <c r="E58" s="7">
         <v>28374.3</v>
       </c>
     </row>
-    <row r="60" spans="3:5" x14ac:dyDescent="0.25">
-      <c r="E60">
-        <f>E58-E59</f>
+    <row r="59" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="E59">
+        <f>E57-E58</f>
         <v>26.75</v>
+      </c>
+    </row>
+    <row r="64" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="E64" t="s">
+        <v>44</v>
+      </c>
+      <c r="F64">
+        <v>696</v>
       </c>
     </row>
     <row r="65" spans="3:6" x14ac:dyDescent="0.25">
       <c r="E65" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F65">
-        <v>696</v>
-      </c>
-    </row>
-    <row r="66" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="E66" t="s">
-        <v>45</v>
-      </c>
-      <c r="F66">
         <v>146</v>
+      </c>
+    </row>
+    <row r="68" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="E68">
+        <v>752.79</v>
+      </c>
+      <c r="F68">
+        <v>26.75</v>
       </c>
     </row>
     <row r="69" spans="3:6" x14ac:dyDescent="0.25">
       <c r="E69">
-        <v>752.79</v>
+        <v>100</v>
       </c>
       <c r="F69">
-        <v>26.75</v>
-      </c>
-    </row>
-    <row r="70" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="E70">
-        <v>100</v>
-      </c>
-      <c r="F70">
-        <f>E70*F69/E69</f>
+        <f>E69*F68/E68</f>
         <v>3.5534478406992656</v>
       </c>
     </row>
-    <row r="75" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C75" s="6" t="s">
+    <row r="74" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C74" s="6" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="77" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C77" s="6" t="s">
+    <row r="76" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C76" s="6" t="s">
         <v>38</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Interfaz para ejecutar SPs y backups de la BDD
</commit_message>
<xml_diff>
--- a/documentacion/SIPRO_TO_DO.xlsx
+++ b/documentacion/SIPRO_TO_DO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PROYECTOS\SIPRO_07\documentacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58923BF5-3B22-40AE-A916-AFB089C80454}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50B1AE48-DE3C-4B2A-A7DC-C5A4938017C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="68">
   <si>
     <t>Implementar registro de acciones</t>
   </si>
@@ -346,6 +346,9 @@
   </si>
   <si>
     <t>Crear funcionalidad de descarga de Ofertas y Demandas a las 4:30</t>
+  </si>
+  <si>
+    <t>Revisar la propuesta_explotacion_vector_precios_bvq.md.. Está implementada la opcion A … pendiente el resto</t>
   </si>
 </sst>
 </file>
@@ -1542,12 +1545,14 @@
         <v>1</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F29" s="3">
         <v>46285</v>
       </c>
-      <c r="G29" s="2"/>
+      <c r="G29" s="3">
+        <v>46299</v>
+      </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="2">
@@ -1605,12 +1610,14 @@
         <v>1</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F32" s="3">
         <v>46285</v>
       </c>
-      <c r="G32" s="2"/>
+      <c r="G32" s="3">
+        <v>46299</v>
+      </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="2">
@@ -1653,6 +1660,11 @@
         <v>46293</v>
       </c>
       <c r="G34" s="2"/>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C35" s="6" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="57" spans="3:6" x14ac:dyDescent="0.25">
       <c r="E57">

</xml_diff>

<commit_message>
Actualizacion de indicadores cuando se produce una venta de acciones
</commit_message>
<xml_diff>
--- a/documentacion/SIPRO_TO_DO.xlsx
+++ b/documentacion/SIPRO_TO_DO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PROYECTOS\SIPRO_07\documentacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50B1AE48-DE3C-4B2A-A7DC-C5A4938017C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E219FD8-9057-427C-8CD3-87DCB9F83072}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Hoja2" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$G$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$G$36</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="71">
   <si>
     <t>Implementar registro de acciones</t>
   </si>
@@ -349,6 +349,15 @@
   </si>
   <si>
     <t>Revisar la propuesta_explotacion_vector_precios_bvq.md.. Está implementada la opcion A … pendiente el resto</t>
+  </si>
+  <si>
+    <t>Actualizar el limpiador de textos, que las frases completas vayan al inicio</t>
+  </si>
+  <si>
+    <t>VectorPrecios</t>
+  </si>
+  <si>
+    <t>Cleaner</t>
   </si>
 </sst>
 </file>
@@ -442,7 +451,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -472,6 +481,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -898,6 +908,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:G76"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -932,7 +943,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -955,7 +966,7 @@
         <v>46194</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -978,7 +989,7 @@
         <v>46207</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -1022,7 +1033,7 @@
       </c>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -1045,7 +1056,7 @@
         <v>46207</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -1068,7 +1079,7 @@
         <v>46249</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -1089,7 +1100,7 @@
       </c>
       <c r="G8" s="2"/>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -1110,7 +1121,7 @@
       </c>
       <c r="G9" s="2"/>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -1154,7 +1165,7 @@
       </c>
       <c r="G11" s="2"/>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -1177,7 +1188,7 @@
         <v>46200</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>12</v>
       </c>
@@ -1200,7 +1211,7 @@
         <v>46207</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>13</v>
       </c>
@@ -1223,7 +1234,7 @@
         <v>46207</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>14</v>
       </c>
@@ -1246,7 +1257,7 @@
         <v>46249</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>15</v>
       </c>
@@ -1269,7 +1280,7 @@
         <v>46207</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <v>16</v>
       </c>
@@ -1313,7 +1324,7 @@
       </c>
       <c r="G18" s="2"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
         <v>18</v>
       </c>
@@ -1336,7 +1347,7 @@
         <v>46249</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
         <v>19</v>
       </c>
@@ -1380,7 +1391,7 @@
       </c>
       <c r="G21" s="2"/>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2">
         <v>21</v>
       </c>
@@ -1403,7 +1414,7 @@
         <v>46250</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2">
         <v>22</v>
       </c>
@@ -1531,7 +1542,7 @@
       </c>
       <c r="G28" s="2"/>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2">
         <v>28</v>
       </c>
@@ -1596,7 +1607,7 @@
       </c>
       <c r="G31" s="2"/>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" s="2">
         <v>31</v>
       </c>
@@ -1662,9 +1673,46 @@
       <c r="G34" s="2"/>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C35" s="6" t="s">
+      <c r="A35" s="13">
+        <v>34</v>
+      </c>
+      <c r="B35" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="C35" s="5" t="s">
         <v>67</v>
       </c>
+      <c r="D35" s="2">
+        <v>1</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F35" s="3">
+        <v>46307</v>
+      </c>
+      <c r="G35" s="2"/>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A36" s="13">
+        <v>35</v>
+      </c>
+      <c r="B36" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="C36" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="D36" s="2">
+        <v>1</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F36" s="3">
+        <v>46307</v>
+      </c>
+      <c r="G36" s="2"/>
     </row>
     <row r="57" spans="3:6" x14ac:dyDescent="0.25">
       <c r="E57">
@@ -1727,6 +1775,13 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:G36" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="4">
+      <filters>
+        <filter val="Pendiente"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <hyperlinks>
     <hyperlink ref="C31" r:id="rId1" xr:uid="{3C22A885-07EB-43DB-A866-EAD7FAA5DC07}"/>
   </hyperlinks>

</xml_diff>

<commit_message>
Seleccion multiple de propietarios para preparar el reporte de patrimonio SRI
</commit_message>
<xml_diff>
--- a/documentacion/SIPRO_TO_DO.xlsx
+++ b/documentacion/SIPRO_TO_DO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PROYECTOS\SIPRO_07\documentacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E219FD8-9057-427C-8CD3-87DCB9F83072}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D006FF2-AD8C-49DA-B33E-B20AAB57B437}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -451,7 +451,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -481,7 +481,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -917,7 +916,7 @@
     <col min="3" max="3" width="133.5703125" style="6" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="17.140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="10" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -1673,10 +1672,10 @@
       <c r="G34" s="2"/>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A35" s="13">
+      <c r="A35" s="2">
         <v>34</v>
       </c>
-      <c r="B35" s="13" t="s">
+      <c r="B35" s="2" t="s">
         <v>69</v>
       </c>
       <c r="C35" s="5" t="s">
@@ -1694,10 +1693,10 @@
       <c r="G35" s="2"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A36" s="13">
+      <c r="A36" s="2">
         <v>35</v>
       </c>
-      <c r="B36" s="13" t="s">
+      <c r="B36" s="2" t="s">
         <v>70</v>
       </c>
       <c r="C36" s="5" t="s">
@@ -1707,12 +1706,14 @@
         <v>1</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F36" s="3">
         <v>46307</v>
       </c>
-      <c r="G36" s="2"/>
+      <c r="G36" s="3">
+        <v>46309</v>
+      </c>
     </row>
     <row r="57" spans="3:6" x14ac:dyDescent="0.25">
       <c r="E57">

</xml_diff>

<commit_message>
Se mejora la actualizacion de ventas de notas de credito
</commit_message>
<xml_diff>
--- a/documentacion/SIPRO_TO_DO.xlsx
+++ b/documentacion/SIPRO_TO_DO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PROYECTOS\SIPRO_07\documentacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D006FF2-AD8C-49DA-B33E-B20AAB57B437}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB3FB19E-4B44-4E66-9C14-52109B458379}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -916,7 +916,7 @@
     <col min="3" max="3" width="133.5703125" style="6" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="17.140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -1302,7 +1302,7 @@
         <v>46256</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
         <v>17</v>
       </c>
@@ -1316,12 +1316,14 @@
         <v>1</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F18" s="3">
         <v>46204</v>
       </c>
-      <c r="G18" s="2"/>
+      <c r="G18" s="3">
+        <v>46322</v>
+      </c>
     </row>
     <row r="19" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
@@ -1369,7 +1371,7 @@
         <v>46249</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="75" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" ht="75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2">
         <v>20</v>
       </c>
@@ -1383,12 +1385,14 @@
         <v>1</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F21" s="3">
         <v>46249</v>
       </c>
-      <c r="G21" s="2"/>
+      <c r="G21" s="3">
+        <v>46322</v>
+      </c>
     </row>
     <row r="22" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2">
@@ -1436,7 +1440,7 @@
         <v>46250</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2">
         <v>23</v>
       </c>
@@ -1450,14 +1454,16 @@
         <v>1</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F24" s="3">
         <v>46249</v>
       </c>
-      <c r="G24" s="2"/>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G24" s="3">
+        <v>46322</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2">
         <v>24</v>
       </c>
@@ -1471,12 +1477,14 @@
         <v>1</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F25" s="3">
         <v>46249</v>
       </c>
-      <c r="G25" s="2"/>
+      <c r="G25" s="3">
+        <v>46322</v>
+      </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="2">
@@ -1671,7 +1679,7 @@
       </c>
       <c r="G34" s="2"/>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" s="2">
         <v>34</v>
       </c>
@@ -1685,14 +1693,16 @@
         <v>1</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F35" s="3">
         <v>46307</v>
       </c>
-      <c r="G35" s="2"/>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="G35" s="3">
+        <v>46309</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" s="2">
         <v>35</v>
       </c>

</xml_diff>